<commit_message>
Se crea la app de acp y kmeans
</commit_message>
<xml_diff>
--- a/ML_Finanzas/Notas/ML_Econ_y_Finan.xlsx
+++ b/ML_Finanzas/Notas/ML_Econ_y_Finan.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CEF754-4A6E-4DC2-87CE-C8D84D2C5886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65E6AAEA-2496-4A13-8A70-5C82D4A12CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43095" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reporteNotas" sheetId="1" r:id="rId1"/>
+    <sheet name="reporteNotas (2)" sheetId="2" r:id="rId2"/>
+    <sheet name="reporteNotas (3)" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'reporteNotas (2)'!$H$1:$J$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'reporteNotas (3)'!$H$1:$J$23</definedName>
+    <definedName name="JR_PAGE_ANCHOR_0_1" localSheetId="1">'reporteNotas (2)'!#REF!</definedName>
+    <definedName name="JR_PAGE_ANCHOR_0_1" localSheetId="2">'reporteNotas (3)'!#REF!</definedName>
     <definedName name="JR_PAGE_ANCHOR_0_1">reporteNotas!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -31,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="58">
   <si>
     <t>NO.</t>
   </si>
@@ -199,6 +205,12 @@
   </si>
   <si>
     <t>Definitiva Corte 1</t>
+  </si>
+  <si>
+    <t>Taller 5</t>
+  </si>
+  <si>
+    <t>Taller 6</t>
   </si>
 </sst>
 </file>
@@ -393,12 +405,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -422,6 +428,12 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -769,12 +781,12 @@
     <col min="5" max="5" width="1.77734375" customWidth="1"/>
     <col min="6" max="6" width="9.33203125" customWidth="1"/>
     <col min="7" max="7" width="0.109375" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="12" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" style="10" customWidth="1"/>
     <col min="9" max="12" width="8.44140625" customWidth="1"/>
     <col min="13" max="16" width="5.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="58.2" thickBot="1">
+    <row r="1" spans="1:16" ht="29.4" thickBot="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -784,29 +796,29 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="11" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="L1" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="M1" s="10"/>
-      <c r="N1" s="10"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
     </row>
@@ -814,36 +826,36 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="11">
-        <v>5</v>
-      </c>
-      <c r="I2" s="10">
+      <c r="D2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="9">
+        <v>5</v>
+      </c>
+      <c r="I2" s="8">
         <v>4.5999999999999996</v>
       </c>
-      <c r="J2" s="10">
-        <v>5</v>
-      </c>
-      <c r="K2" s="10">
-        <v>3</v>
-      </c>
-      <c r="L2" s="13">
+      <c r="J2" s="8">
+        <v>5</v>
+      </c>
+      <c r="K2" s="8">
+        <v>3</v>
+      </c>
+      <c r="L2" s="11">
         <f>+I2*0.6+AVERAGE(H2,J2:K2)*0.4</f>
         <v>4.4933333333333332</v>
       </c>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
       <c r="O2" s="1"/>
       <c r="P2" s="1"/>
     </row>
@@ -857,30 +869,30 @@
       <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="11">
-        <v>5</v>
-      </c>
-      <c r="I3" s="10">
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="9">
+        <v>5</v>
+      </c>
+      <c r="I3" s="8">
         <v>4.7</v>
       </c>
-      <c r="J3" s="10">
-        <v>5</v>
-      </c>
-      <c r="K3" s="10">
-        <v>5</v>
-      </c>
-      <c r="L3" s="13">
+      <c r="J3" s="8">
+        <v>5</v>
+      </c>
+      <c r="K3" s="8">
+        <v>5</v>
+      </c>
+      <c r="L3" s="11">
         <f t="shared" ref="L3:L23" si="0">+I3*0.6+AVERAGE(H3,J3:K3)*0.4</f>
         <v>4.82</v>
       </c>
-      <c r="M3" s="10"/>
-      <c r="N3" s="10"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
       <c r="O3" s="1"/>
       <c r="P3" s="1"/>
     </row>
@@ -894,30 +906,30 @@
       <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="11">
-        <v>5</v>
-      </c>
-      <c r="I4" s="10">
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="9">
+        <v>5</v>
+      </c>
+      <c r="I4" s="8">
         <v>4.5</v>
       </c>
-      <c r="J4" s="10">
-        <v>5</v>
-      </c>
-      <c r="K4" s="10">
-        <v>5</v>
-      </c>
-      <c r="L4" s="13">
+      <c r="J4" s="8">
+        <v>5</v>
+      </c>
+      <c r="K4" s="8">
+        <v>5</v>
+      </c>
+      <c r="L4" s="11">
         <f t="shared" si="0"/>
         <v>4.6999999999999993</v>
       </c>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
     </row>
@@ -931,30 +943,30 @@
       <c r="C5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="11">
-        <v>1</v>
-      </c>
-      <c r="I5" s="10">
-        <v>1</v>
-      </c>
-      <c r="J5" s="10">
-        <v>1</v>
-      </c>
-      <c r="K5" s="10">
-        <v>5</v>
-      </c>
-      <c r="L5" s="13">
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1</v>
+      </c>
+      <c r="J5" s="8">
+        <v>1</v>
+      </c>
+      <c r="K5" s="8">
+        <v>5</v>
+      </c>
+      <c r="L5" s="11">
         <f t="shared" si="0"/>
         <v>1.5333333333333334</v>
       </c>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
     </row>
@@ -968,30 +980,30 @@
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="11">
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="9">
         <v>4</v>
       </c>
-      <c r="I6" s="10">
+      <c r="I6" s="8">
         <v>3.5</v>
       </c>
-      <c r="J6" s="10">
-        <v>1</v>
-      </c>
-      <c r="K6" s="10">
+      <c r="J6" s="8">
+        <v>1</v>
+      </c>
+      <c r="K6" s="8">
         <v>4.5</v>
       </c>
-      <c r="L6" s="13">
+      <c r="L6" s="11">
         <f t="shared" si="0"/>
         <v>3.3666666666666667</v>
       </c>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
@@ -1005,30 +1017,30 @@
       <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="11">
-        <v>5</v>
-      </c>
-      <c r="I7" s="10">
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="9">
+        <v>5</v>
+      </c>
+      <c r="I7" s="8">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J7" s="10">
-        <v>5</v>
-      </c>
-      <c r="K7" s="10">
-        <v>5</v>
-      </c>
-      <c r="L7" s="13">
+      <c r="J7" s="8">
+        <v>5</v>
+      </c>
+      <c r="K7" s="8">
+        <v>5</v>
+      </c>
+      <c r="L7" s="11">
         <f t="shared" si="0"/>
         <v>4.9399999999999995</v>
       </c>
-      <c r="M7" s="10"/>
-      <c r="N7" s="10"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
       <c r="O7" s="1"/>
       <c r="P7" s="1"/>
     </row>
@@ -1042,30 +1054,30 @@
       <c r="C8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="11">
-        <v>5</v>
-      </c>
-      <c r="I8" s="10">
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="9">
+        <v>5</v>
+      </c>
+      <c r="I8" s="8">
         <v>4.3</v>
       </c>
-      <c r="J8" s="10">
-        <v>5</v>
-      </c>
-      <c r="K8" s="10">
-        <v>5</v>
-      </c>
-      <c r="L8" s="13">
+      <c r="J8" s="8">
+        <v>5</v>
+      </c>
+      <c r="K8" s="8">
+        <v>5</v>
+      </c>
+      <c r="L8" s="11">
         <f t="shared" si="0"/>
         <v>4.58</v>
       </c>
-      <c r="M8" s="10"/>
-      <c r="N8" s="10"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
     </row>
@@ -1079,30 +1091,30 @@
       <c r="C9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="11">
-        <v>5</v>
-      </c>
-      <c r="I9" s="10">
-        <v>5</v>
-      </c>
-      <c r="J9" s="10">
-        <v>5</v>
-      </c>
-      <c r="K9" s="10">
-        <v>1</v>
-      </c>
-      <c r="L9" s="13">
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="9">
+        <v>5</v>
+      </c>
+      <c r="I9" s="8">
+        <v>5</v>
+      </c>
+      <c r="J9" s="8">
+        <v>5</v>
+      </c>
+      <c r="K9" s="8">
+        <v>1</v>
+      </c>
+      <c r="L9" s="11">
         <f t="shared" si="0"/>
         <v>4.4666666666666668</v>
       </c>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
     </row>
@@ -1116,30 +1128,30 @@
       <c r="C10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="11">
-        <v>5</v>
-      </c>
-      <c r="I10" s="10">
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="9">
+        <v>5</v>
+      </c>
+      <c r="I10" s="8">
         <v>4.8</v>
       </c>
-      <c r="J10" s="10">
-        <v>5</v>
-      </c>
-      <c r="K10" s="10">
-        <v>5</v>
-      </c>
-      <c r="L10" s="13">
+      <c r="J10" s="8">
+        <v>5</v>
+      </c>
+      <c r="K10" s="8">
+        <v>5</v>
+      </c>
+      <c r="L10" s="11">
         <f t="shared" si="0"/>
         <v>4.88</v>
       </c>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
     </row>
@@ -1153,30 +1165,30 @@
       <c r="C11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="11">
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="9">
         <v>4</v>
       </c>
-      <c r="I11" s="10">
+      <c r="I11" s="8">
         <v>4.7</v>
       </c>
-      <c r="J11" s="10">
-        <v>1</v>
-      </c>
-      <c r="K11" s="10">
-        <v>5</v>
-      </c>
-      <c r="L11" s="13">
+      <c r="J11" s="8">
+        <v>1</v>
+      </c>
+      <c r="K11" s="8">
+        <v>5</v>
+      </c>
+      <c r="L11" s="11">
         <f t="shared" si="0"/>
         <v>4.1533333333333333</v>
       </c>
-      <c r="M11" s="10"/>
-      <c r="N11" s="10"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
       <c r="O11" s="1"/>
       <c r="P11" s="1"/>
     </row>
@@ -1190,30 +1202,30 @@
       <c r="C12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="11">
-        <v>5</v>
-      </c>
-      <c r="I12" s="10">
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="9">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8">
         <v>4.7</v>
       </c>
-      <c r="J12" s="10">
-        <v>5</v>
-      </c>
-      <c r="K12" s="10">
-        <v>5</v>
-      </c>
-      <c r="L12" s="13">
+      <c r="J12" s="8">
+        <v>5</v>
+      </c>
+      <c r="K12" s="8">
+        <v>5</v>
+      </c>
+      <c r="L12" s="11">
         <f t="shared" si="0"/>
         <v>4.82</v>
       </c>
-      <c r="M12" s="10"/>
-      <c r="N12" s="10"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
       <c r="O12" s="1"/>
       <c r="P12" s="1"/>
     </row>
@@ -1227,30 +1239,30 @@
       <c r="C13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="11">
-        <v>1</v>
-      </c>
-      <c r="I13" s="10">
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="9">
+        <v>1</v>
+      </c>
+      <c r="I13" s="8">
         <v>4.5</v>
       </c>
-      <c r="J13" s="10">
-        <v>5</v>
-      </c>
-      <c r="K13" s="10">
-        <v>5</v>
-      </c>
-      <c r="L13" s="13">
+      <c r="J13" s="8">
+        <v>5</v>
+      </c>
+      <c r="K13" s="8">
+        <v>5</v>
+      </c>
+      <c r="L13" s="11">
         <f t="shared" si="0"/>
         <v>4.1666666666666661</v>
       </c>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
       <c r="O13" s="1"/>
       <c r="P13" s="1"/>
     </row>
@@ -1264,30 +1276,30 @@
       <c r="C14" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="11">
-        <v>5</v>
-      </c>
-      <c r="I14" s="10">
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="9">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8">
         <v>4</v>
       </c>
-      <c r="J14" s="10">
-        <v>5</v>
-      </c>
-      <c r="K14" s="10">
-        <v>5</v>
-      </c>
-      <c r="L14" s="13">
+      <c r="J14" s="8">
+        <v>5</v>
+      </c>
+      <c r="K14" s="8">
+        <v>5</v>
+      </c>
+      <c r="L14" s="11">
         <f t="shared" si="0"/>
         <v>4.4000000000000004</v>
       </c>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
       <c r="O14" s="1"/>
       <c r="P14" s="1"/>
     </row>
@@ -1301,30 +1313,30 @@
       <c r="C15" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="11">
-        <v>5</v>
-      </c>
-      <c r="I15" s="10">
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="9">
+        <v>5</v>
+      </c>
+      <c r="I15" s="8">
         <v>4.5999999999999996</v>
       </c>
-      <c r="J15" s="10">
-        <v>1</v>
-      </c>
-      <c r="K15" s="10">
-        <v>5</v>
-      </c>
-      <c r="L15" s="13">
+      <c r="J15" s="8">
+        <v>1</v>
+      </c>
+      <c r="K15" s="8">
+        <v>5</v>
+      </c>
+      <c r="L15" s="11">
         <f t="shared" si="0"/>
         <v>4.2266666666666666</v>
       </c>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
       <c r="O15" s="1"/>
       <c r="P15" s="1"/>
     </row>
@@ -1338,30 +1350,30 @@
       <c r="C16" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="11">
-        <v>5</v>
-      </c>
-      <c r="I16" s="10">
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="9">
+        <v>5</v>
+      </c>
+      <c r="I16" s="8">
         <v>4.9000000000000004</v>
       </c>
-      <c r="J16" s="10">
-        <v>5</v>
-      </c>
-      <c r="K16" s="10">
-        <v>5</v>
-      </c>
-      <c r="L16" s="13">
+      <c r="J16" s="8">
+        <v>5</v>
+      </c>
+      <c r="K16" s="8">
+        <v>5</v>
+      </c>
+      <c r="L16" s="11">
         <f t="shared" si="0"/>
         <v>4.9399999999999995</v>
       </c>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
       <c r="O16" s="1"/>
       <c r="P16" s="1"/>
     </row>
@@ -1375,30 +1387,30 @@
       <c r="C17" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="11">
-        <v>5</v>
-      </c>
-      <c r="I17" s="10">
-        <v>5</v>
-      </c>
-      <c r="J17" s="10">
-        <v>5</v>
-      </c>
-      <c r="K17" s="10">
-        <v>5</v>
-      </c>
-      <c r="L17" s="13">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="9">
+        <v>5</v>
+      </c>
+      <c r="I17" s="8">
+        <v>5</v>
+      </c>
+      <c r="J17" s="8">
+        <v>5</v>
+      </c>
+      <c r="K17" s="8">
+        <v>5</v>
+      </c>
+      <c r="L17" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
     </row>
@@ -1412,30 +1424,30 @@
       <c r="C18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="11">
-        <v>5</v>
-      </c>
-      <c r="I18" s="10">
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="9">
+        <v>5</v>
+      </c>
+      <c r="I18" s="8">
         <v>4.3</v>
       </c>
-      <c r="J18" s="10">
-        <v>5</v>
-      </c>
-      <c r="K18" s="10">
-        <v>5</v>
-      </c>
-      <c r="L18" s="13">
+      <c r="J18" s="8">
+        <v>5</v>
+      </c>
+      <c r="K18" s="8">
+        <v>5</v>
+      </c>
+      <c r="L18" s="11">
         <f t="shared" si="0"/>
         <v>4.58</v>
       </c>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
       <c r="O18" s="1"/>
       <c r="P18" s="1"/>
     </row>
@@ -1449,30 +1461,30 @@
       <c r="C19" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="11">
-        <v>5</v>
-      </c>
-      <c r="I19" s="10">
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="9">
+        <v>5</v>
+      </c>
+      <c r="I19" s="8">
         <v>4.5</v>
       </c>
-      <c r="J19" s="10">
-        <v>5</v>
-      </c>
-      <c r="K19" s="10">
-        <v>5</v>
-      </c>
-      <c r="L19" s="13">
+      <c r="J19" s="8">
+        <v>5</v>
+      </c>
+      <c r="K19" s="8">
+        <v>5</v>
+      </c>
+      <c r="L19" s="11">
         <f t="shared" si="0"/>
         <v>4.6999999999999993</v>
       </c>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
       <c r="O19" s="1"/>
       <c r="P19" s="1"/>
     </row>
@@ -1486,30 +1498,30 @@
       <c r="C20" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="11">
-        <v>5</v>
-      </c>
-      <c r="I20" s="10">
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="9">
+        <v>5</v>
+      </c>
+      <c r="I20" s="8">
         <v>4</v>
       </c>
-      <c r="J20" s="10">
-        <v>5</v>
-      </c>
-      <c r="K20" s="10">
-        <v>5</v>
-      </c>
-      <c r="L20" s="13">
+      <c r="J20" s="8">
+        <v>5</v>
+      </c>
+      <c r="K20" s="8">
+        <v>5</v>
+      </c>
+      <c r="L20" s="11">
         <f t="shared" si="0"/>
         <v>4.4000000000000004</v>
       </c>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
       <c r="O20" s="1"/>
       <c r="P20" s="1"/>
     </row>
@@ -1523,30 +1535,30 @@
       <c r="C21" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="E21" s="6"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="11">
-        <v>5</v>
-      </c>
-      <c r="I21" s="10">
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="9">
+        <v>5</v>
+      </c>
+      <c r="I21" s="8">
         <v>4.7</v>
       </c>
-      <c r="J21" s="10">
-        <v>5</v>
-      </c>
-      <c r="K21" s="10">
-        <v>5</v>
-      </c>
-      <c r="L21" s="13">
+      <c r="J21" s="8">
+        <v>5</v>
+      </c>
+      <c r="K21" s="8">
+        <v>5</v>
+      </c>
+      <c r="L21" s="11">
         <f t="shared" si="0"/>
         <v>4.82</v>
       </c>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
       <c r="O21" s="1"/>
       <c r="P21" s="1"/>
     </row>
@@ -1560,30 +1572,30 @@
       <c r="C22" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="11">
-        <v>5</v>
-      </c>
-      <c r="I22" s="10">
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="9">
+        <v>5</v>
+      </c>
+      <c r="I22" s="8">
         <v>4.8</v>
       </c>
-      <c r="J22" s="10">
-        <v>5</v>
-      </c>
-      <c r="K22" s="10">
-        <v>5</v>
-      </c>
-      <c r="L22" s="13">
+      <c r="J22" s="8">
+        <v>5</v>
+      </c>
+      <c r="K22" s="8">
+        <v>5</v>
+      </c>
+      <c r="L22" s="11">
         <f t="shared" si="0"/>
         <v>4.88</v>
       </c>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
       <c r="O22" s="1"/>
       <c r="P22" s="1"/>
     </row>
@@ -1597,61 +1609,1585 @@
       <c r="C23" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="11">
-        <v>5</v>
-      </c>
-      <c r="I23" s="10">
-        <v>5</v>
-      </c>
-      <c r="J23" s="10">
-        <v>5</v>
-      </c>
-      <c r="K23" s="10">
-        <v>5</v>
-      </c>
-      <c r="L23" s="13">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="9">
+        <v>5</v>
+      </c>
+      <c r="I23" s="8">
+        <v>5</v>
+      </c>
+      <c r="J23" s="8">
+        <v>5</v>
+      </c>
+      <c r="K23" s="8">
+        <v>5</v>
+      </c>
+      <c r="L23" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
       <c r="O23" s="1"/>
       <c r="P23" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D14:F14"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="D21:F21"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="D1:F1"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DB7F907-F15A-4382-9C91-D4A812A0D9EE}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="1.77734375" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="0.109375" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" style="10" customWidth="1"/>
+    <col min="9" max="10" width="8.44140625" customWidth="1"/>
+    <col min="11" max="14" width="5.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="29.4" thickBot="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="I2" s="8">
+        <v>1</v>
+      </c>
+      <c r="J2" s="11">
+        <f>AVERAGE(H2:I2)</f>
+        <v>2.25</v>
+      </c>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="9">
+        <v>5</v>
+      </c>
+      <c r="I3" s="8">
+        <v>5</v>
+      </c>
+      <c r="J3" s="11">
+        <f t="shared" ref="J3:J23" si="0">AVERAGE(H3:I3)</f>
+        <v>5</v>
+      </c>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+    </row>
+    <row r="4" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="9">
+        <v>5</v>
+      </c>
+      <c r="I4" s="8">
+        <v>5</v>
+      </c>
+      <c r="J4" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+    </row>
+    <row r="5" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="8">
+        <v>5</v>
+      </c>
+      <c r="J5" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+    </row>
+    <row r="6" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>5</v>
+      </c>
+      <c r="J6" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+    </row>
+    <row r="7" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="9">
+        <v>1</v>
+      </c>
+      <c r="I7" s="8">
+        <v>5</v>
+      </c>
+      <c r="J7" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+    </row>
+    <row r="8" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="9">
+        <v>1</v>
+      </c>
+      <c r="I8" s="8">
+        <v>5</v>
+      </c>
+      <c r="J8" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+    </row>
+    <row r="9" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="9">
+        <v>5</v>
+      </c>
+      <c r="I9" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="J9" s="11">
+        <f t="shared" si="0"/>
+        <v>4.75</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+    </row>
+    <row r="10" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="9">
+        <v>5</v>
+      </c>
+      <c r="I10" s="8">
+        <v>5</v>
+      </c>
+      <c r="J10" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+    </row>
+    <row r="11" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="9">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8">
+        <v>5</v>
+      </c>
+      <c r="J11" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="9">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8">
+        <v>5</v>
+      </c>
+      <c r="J12" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="9">
+        <v>1</v>
+      </c>
+      <c r="I13" s="8">
+        <v>5</v>
+      </c>
+      <c r="J13" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="9">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8">
+        <v>5</v>
+      </c>
+      <c r="J14" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+    </row>
+    <row r="15" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="9">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8">
+        <v>5</v>
+      </c>
+      <c r="J15" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="9">
+        <v>5</v>
+      </c>
+      <c r="I16">
+        <v>5</v>
+      </c>
+      <c r="J16" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+    </row>
+    <row r="17" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="9">
+        <v>5</v>
+      </c>
+      <c r="I17" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="J17" s="11">
+        <f t="shared" si="0"/>
+        <v>4.75</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="9">
+        <v>1</v>
+      </c>
+      <c r="I18" s="8">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+    </row>
+    <row r="19" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="9">
+        <v>5</v>
+      </c>
+      <c r="I19" s="8">
+        <v>5</v>
+      </c>
+      <c r="J19" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+    </row>
+    <row r="20" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="9">
+        <v>5</v>
+      </c>
+      <c r="I20" s="8">
+        <v>5</v>
+      </c>
+      <c r="J20" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+    </row>
+    <row r="21" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="9">
+        <v>5</v>
+      </c>
+      <c r="I21" s="8">
+        <v>5</v>
+      </c>
+      <c r="J21" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+    </row>
+    <row r="22" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="9">
+        <v>5</v>
+      </c>
+      <c r="I22" s="8">
+        <v>5</v>
+      </c>
+      <c r="J22" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+    </row>
+    <row r="23" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="9">
+        <v>5</v>
+      </c>
+      <c r="I23" s="8">
+        <v>5</v>
+      </c>
+      <c r="J23" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D6:F6"/>
+  </mergeCells>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCEAF046-B3AA-47D8-AEAE-90675772F06D}">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:N23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="21.77734375" customWidth="1"/>
+    <col min="5" max="5" width="1.77734375" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" customWidth="1"/>
+    <col min="7" max="7" width="0.109375" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" style="10" customWidth="1"/>
+    <col min="9" max="10" width="8.44140625" customWidth="1"/>
+    <col min="11" max="14" width="5.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="29.4" thickBot="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="9">
+        <v>3.5</v>
+      </c>
+      <c r="I2" s="8">
+        <v>1</v>
+      </c>
+      <c r="J2" s="11">
+        <f>AVERAGE(H2:I2)</f>
+        <v>2.25</v>
+      </c>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="9">
+        <v>5</v>
+      </c>
+      <c r="I3" s="8">
+        <v>5</v>
+      </c>
+      <c r="J3" s="11">
+        <f t="shared" ref="J3:J23" si="0">AVERAGE(H3:I3)</f>
+        <v>5</v>
+      </c>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+    </row>
+    <row r="4" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="9">
+        <v>5</v>
+      </c>
+      <c r="I4" s="8">
+        <v>5</v>
+      </c>
+      <c r="J4" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+    </row>
+    <row r="5" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="8">
+        <v>5</v>
+      </c>
+      <c r="J5" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+    </row>
+    <row r="6" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="8">
+        <v>5</v>
+      </c>
+      <c r="J6" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+    </row>
+    <row r="7" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A7" s="3">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="9">
+        <v>1</v>
+      </c>
+      <c r="I7" s="8">
+        <v>5</v>
+      </c>
+      <c r="J7" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+    </row>
+    <row r="8" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="9">
+        <v>1</v>
+      </c>
+      <c r="I8" s="8">
+        <v>5</v>
+      </c>
+      <c r="J8" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+    </row>
+    <row r="9" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A9" s="3">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="9">
+        <v>5</v>
+      </c>
+      <c r="I9" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="J9" s="11">
+        <f t="shared" si="0"/>
+        <v>4.75</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+    </row>
+    <row r="10" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A10" s="3">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="9">
+        <v>5</v>
+      </c>
+      <c r="I10" s="8">
+        <v>5</v>
+      </c>
+      <c r="J10" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+    </row>
+    <row r="11" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A11" s="3">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="9">
+        <v>1</v>
+      </c>
+      <c r="I11" s="8">
+        <v>5</v>
+      </c>
+      <c r="J11" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A12" s="3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="9">
+        <v>5</v>
+      </c>
+      <c r="I12" s="8">
+        <v>5</v>
+      </c>
+      <c r="J12" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A13" s="3">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="9">
+        <v>1</v>
+      </c>
+      <c r="I13" s="8">
+        <v>5</v>
+      </c>
+      <c r="J13" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+    </row>
+    <row r="14" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A14" s="3">
+        <v>13</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="9">
+        <v>5</v>
+      </c>
+      <c r="I14" s="8">
+        <v>5</v>
+      </c>
+      <c r="J14" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+    </row>
+    <row r="15" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A15" s="3">
+        <v>14</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="9">
+        <v>1</v>
+      </c>
+      <c r="I15" s="8">
+        <v>5</v>
+      </c>
+      <c r="J15" s="11">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+    </row>
+    <row r="16" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A16" s="3">
+        <v>15</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="9">
+        <v>5</v>
+      </c>
+      <c r="I16">
+        <v>5</v>
+      </c>
+      <c r="J16" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+    </row>
+    <row r="17" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A17" s="3">
+        <v>16</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="9">
+        <v>5</v>
+      </c>
+      <c r="I17" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="J17" s="11">
+        <f t="shared" si="0"/>
+        <v>4.75</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A18" s="3">
+        <v>17</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="9">
+        <v>1</v>
+      </c>
+      <c r="I18" s="8">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+    </row>
+    <row r="19" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A19" s="3">
+        <v>18</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="9">
+        <v>5</v>
+      </c>
+      <c r="I19" s="8">
+        <v>5</v>
+      </c>
+      <c r="J19" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+    </row>
+    <row r="20" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A20" s="3">
+        <v>19</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="9">
+        <v>5</v>
+      </c>
+      <c r="I20" s="8">
+        <v>5</v>
+      </c>
+      <c r="J20" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+    </row>
+    <row r="21" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A21" s="3">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="9">
+        <v>5</v>
+      </c>
+      <c r="I21" s="8">
+        <v>5</v>
+      </c>
+      <c r="J21" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+    </row>
+    <row r="22" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A22" s="3">
+        <v>21</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="9">
+        <v>5</v>
+      </c>
+      <c r="I22" s="8">
+        <v>5</v>
+      </c>
+      <c r="J22" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+    </row>
+    <row r="23" spans="1:14" ht="25.05" customHeight="1">
+      <c r="A23" s="3">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="9">
+        <v>5</v>
+      </c>
+      <c r="I23" s="8">
+        <v>5</v>
+      </c>
+      <c r="J23" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="D19:F19"/>
+    <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:F15"/>
+    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D17:F17"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="D2:F2"/>
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D6:F6"/>
+  </mergeCells>
+  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
 </file>
</xml_diff>